<commit_message>
modify the ListMachine return
</commit_message>
<xml_diff>
--- a/Backend/tickets/UploadMachines.xlsx
+++ b/Backend/tickets/UploadMachines.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rani_3yana\M-Iot_Backend\Backend\tickets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2183767C-E1DA-41F9-9546-7F27DA00A000}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF109E09-EBA6-4BB8-AA64-94E41F2CF4E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,9 +109,6 @@
     <t>CAP_IDEN_001</t>
   </si>
   <si>
-    <t>machine_date_installation</t>
-  </si>
-  <si>
     <t>CAP_IDEN_002</t>
   </si>
   <si>
@@ -125,6 +122,9 @@
   </si>
   <si>
     <t>CAP_MACH2_002</t>
+  </si>
+  <si>
+    <t>machine_date_install</t>
   </si>
 </sst>
 </file>
@@ -522,7 +522,7 @@
         <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
         <v>24</v>
@@ -603,7 +603,7 @@
         <v>45882</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
@@ -629,7 +629,7 @@
         <v>45882</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
         <v>7</v>
@@ -655,7 +655,7 @@
         <v>45882</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
         <v>7</v>
@@ -681,7 +681,7 @@
         <v>45882</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
@@ -707,7 +707,7 @@
         <v>45883</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -724,7 +724,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
@@ -733,7 +733,7 @@
         <v>45883</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
         <v>16</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>27</v>
@@ -759,7 +759,7 @@
         <v>45883</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
         <v>16</v>
@@ -776,7 +776,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -785,7 +785,7 @@
         <v>45883</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
         <v>21</v>

</xml_diff>